<commit_message>
Controleer 6BCW-tabellen, OVUR, figuren en evaluatie volgens 5BCW
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Blanco_verslag_6BCW_CONCEPT.xlsx
+++ b/Blanco_verslag_6BCW_CONCEPT.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verslag" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Verslag'!$B$2:$H$79</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Verslag'!$B$2:$H$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -87,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -102,6 +102,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H79"/>
+  <dimension ref="B2:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -842,20 +843,32 @@
     <row r="69" ht="24" customHeight="1">
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>4 · ATTITUDE EN VERZORGING  / 2</t>
+          <t>4 · ATTITUDE EN VERZORGING (productafspraken)  / 2</t>
         </is>
       </c>
     </row>
     <row r="70" ht="22" customHeight="1">
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Groepsbijdrage en taakverdeling</t>
+          <t>Bestandsvorm en termijn</t>
         </is>
       </c>
       <c r="C70" s="6" t="n"/>
     </row>
-    <row r="71" ht="22" customHeight="1"/>
-    <row r="72" ht="22" customHeight="1"/>
+    <row r="71" ht="22" customHeight="1">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Aantoonbaar groepsproduct</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Feedbackblok behouden</t>
+        </is>
+      </c>
+    </row>
     <row r="73" ht="22" customHeight="1">
       <c r="B73" s="3" t="inlineStr">
         <is>
@@ -875,8 +888,84 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="24" customHeight="1">
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>PRODUCTPUNTEN /10 · in te vullen door de leerkracht</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1. Verkennen &amp; onderzoeken</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="10" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2. Onderzoek uitvoeren</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>3</v>
+      </c>
+      <c r="E83" s="10" t="n"/>
+    </row>
+    <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>3. Concluderen</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
+      <c r="E84" s="10" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>4. Attitude en verzorging (product)</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>2</v>
+      </c>
+      <c r="E85" s="10" t="n"/>
+    </row>
+    <row r="86">
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Totaal /10</t>
+        </is>
+      </c>
+      <c r="E86">
+        <f>SUM(E82:E85)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Product 60 % (groepspunt); proces/attitude 40 % (individueel volgens Bijlage C).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Indienen via Smartschool: één week na het labo, uiterlijk 23.59 u; concrete datum/zone vooraf door de leerkracht.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="27">
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="C57:H60"/>
     <mergeCell ref="C73:H77"/>
@@ -888,6 +977,7 @@
     <mergeCell ref="C61:H63"/>
     <mergeCell ref="C64:H67"/>
     <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B81:H81"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="C10:H11"/>
     <mergeCell ref="B27:H27"/>
@@ -896,14 +986,16 @@
     <mergeCell ref="C12:H13"/>
     <mergeCell ref="C47:H50"/>
     <mergeCell ref="C6:H6"/>
+    <mergeCell ref="B88:H88"/>
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="C18:H20"/>
     <mergeCell ref="B69:H69"/>
+    <mergeCell ref="B87:H87"/>
     <mergeCell ref="C51:H54"/>
     <mergeCell ref="B28:H28"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="2" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="3" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Veranker lesdoelen en zes STEM-doelen met doelgerichte evaluatie
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Blanco_verslag_6BCW_CONCEPT.xlsx
+++ b/Blanco_verslag_6BCW_CONCEPT.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verslag" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STEM-doelkaart" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Verslag'!$B$2:$H$88</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'STEM-doelkaart'!$A$1:$F$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +48,11 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -70,7 +77,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -83,11 +90,16 @@
         <color rgb="00B8CEDA"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00B8CEDA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,6 +115,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -998,4 +1017,197 @@
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="3" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="67" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>STEM-DOELKAART 6BCW · bewijs en feedforward (geen extra cijfer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Leerplandoel</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Wat moet je aantonen?</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Verplicht bewijs in deze cursus</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Vindplaats</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Nog niet / op weg / aangetoond</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>Feedback + volgende stap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>1 S</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Een afgebakende vraag en beredeneerde hypothese toetsen met waarnemingen; de methode en conclusie kritisch communiceren.</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Labo 04/07/15/25: vraag, hypothese, data en besluit.</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>2 S</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Metingen noteren met symbool, SI-eenheid, meetnauwkeurigheid, beduidende cijfers en waar zinvol machten van tien.</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Labo 02/09/21/25: symbolen, SI, meetresolutie, beduidende cijfers en machten van tien.</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="13" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>3 S</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Meetinstrumenten en technische systemen nauwkeurig, veilig en duurzaam inzetten; ruwe data controleerbaar bewaren.</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Labo 05/12/21/25: veilige opstelling, betrouwbaar meetbewijs en duurzaam opruimen.</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>4 S</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Voor een concreet probleem een oplossing ontwikkelen met een fysisch én wiskundig model, technische keuzes, test en bijsturing.</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Labo 07: twee opvangontwerpen, model, videotoets en hertoets na bijsturing.</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>5 S</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Bij een maatschappelijke uitdaging wetenschap, technologie en wiskunde én gevolgen voor verschillende betrokkenen afwegen.</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Labo 20: dB-berekening en twee maatschappelijke perspectieven op geluidsbeperking.</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>6 S</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Een volledige onderzoekscyclus uitvoeren: oriëntatie, vraag, methode, data, analyse, conclusie en rapportering.</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Labo 25: alle zeven fasen in plan, ruwe data en poster.</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="13" t="n"/>
+      <c r="F8" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>De docent kent geen zes bonuspunten toe: zie product /10 (60 %) en proces /10 (40 %) in Bijlage B/C.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A10:F10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Maak lesdoelen per leerling aantoonbaar en STEM-evaluatie gericht
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Blanco_verslag_6BCW_CONCEPT.xlsx
+++ b/Blanco_verslag_6BCW_CONCEPT.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Verslag'!$B$2:$H$88</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'STEM-doelkaart'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'STEM-doelkaart'!$A$1:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1025,7 +1025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1202,9 +1202,17 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Kopieer deze doelkaart per leerling. Noteer naam: ……………  ·  De status volgt uit groepsproduct én individuele uitleg/observatie.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>